<commit_message>
Refactor Project Entity Frontend and Docs: project-structure
</commit_message>
<xml_diff>
--- a/project-structure.xlsx
+++ b/project-structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\project\pronaflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30720F47-4E5F-43E4-8F06-A7CEC6934FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EABE46-6F34-4245-946E-856B03541162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="1" xr2:uid="{159F88DC-058F-4C26-BFDD-C91DC9F7BACE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="119">
   <si>
     <t>Hệ thống Tài liệu Kỹ thuật và đặc tả hệ thống</t>
   </si>
@@ -352,6 +352,51 @@
   </si>
   <si>
     <t>Bản ghi khóa phụ thuộc</t>
+  </si>
+  <si>
+    <t>projects/</t>
+  </si>
+  <si>
+    <t>api/</t>
+  </si>
+  <si>
+    <t>ProjectCard/</t>
+  </si>
+  <si>
+    <t>ProjectRow/</t>
+  </si>
+  <si>
+    <t>KanbanColumn/</t>
+  </si>
+  <si>
+    <t>CreateProject/</t>
+  </si>
+  <si>
+    <t>ProjectActions/</t>
+  </si>
+  <si>
+    <t>hooks/</t>
+  </si>
+  <si>
+    <t>UI components đặc thù cho project</t>
+  </si>
+  <si>
+    <t>[Module 3] Quản lý vòng đời dự án</t>
+  </si>
+  <si>
+    <t>Thẻ dự án (Grid View)</t>
+  </si>
+  <si>
+    <t>Dòng dự án (List View)</t>
+  </si>
+  <si>
+    <t>Cột Kanban theo trạng thái Lifecycle</t>
+  </si>
+  <si>
+    <t>From tạo dự án &amp; Template</t>
+  </si>
+  <si>
+    <t>Menu tùy chỉnh (Edit, Delete, Archive)</t>
   </si>
 </sst>
 </file>
@@ -455,7 +500,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -489,6 +534,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -987,18 +1035,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE8C67B-B50C-42D4-8C38-F0CBF607944D}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.69921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="14" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="11.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="36.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="83.5" style="19" customWidth="1"/>
+    <col min="6" max="8" width="11.5" style="14" customWidth="1"/>
+    <col min="9" max="9" width="36.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="83.5" style="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1010,8 +1059,11 @@
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1023,8 +1075,11 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1036,8 +1091,11 @@
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1049,8 +1107,11 @@
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
@@ -1060,582 +1121,872 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="I7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="J7" s="19" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
-      <c r="C9" s="16" t="s">
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="17"/>
+      <c r="C9" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="16"/>
-      <c r="C10" s="16" t="s">
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="17"/>
+      <c r="C10" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" t="s">
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="20"/>
-    </row>
-    <row r="11" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="J10" s="21"/>
+    </row>
+    <row r="11" spans="1:10" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A11" s="14"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="16" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="16"/>
-      <c r="F11" t="s">
+      <c r="E11" s="17"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" t="s">
         <v>66</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="J11" s="21" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="14"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="16" t="s">
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="16"/>
-      <c r="F12" t="s">
+      <c r="E12" s="17"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="J12" s="21" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="14"/>
-      <c r="B13" s="17"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="9"/>
       <c r="D13" s="10"/>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="G13" s="20"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="J13" s="21"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
-      <c r="B14" s="17"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="9"/>
       <c r="D14" s="10"/>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="G14" s="20"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="J14" s="21"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="14"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="16" t="s">
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" t="s">
+      <c r="E15" s="17"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" t="s">
         <v>88</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="J15" s="21" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="14"/>
-      <c r="B16" s="17"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="9"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="G16" s="20"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="J16" s="21"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="14"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="16" t="s">
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="16"/>
-      <c r="G17" s="20"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="17"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="J17" s="21"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="16" t="s">
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="16"/>
-      <c r="F18" t="s">
+      <c r="E18" s="17"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" t="s">
         <v>89</v>
       </c>
-      <c r="G18" s="20"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J18" s="21"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="16" t="s">
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="16"/>
-      <c r="F19" t="s">
+      <c r="E19" s="17"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" t="s">
         <v>90</v>
       </c>
-      <c r="G19" s="20"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J19" s="21"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="16" t="s">
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="16"/>
-      <c r="F20" t="s">
+      <c r="E20" s="17"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="20"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="16"/>
-      <c r="C21" s="16" t="s">
+      <c r="J20" s="21"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" t="s">
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" t="s">
         <v>76</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="J21" s="21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="16"/>
-      <c r="F22" t="s">
+      <c r="E22" s="17"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" t="s">
         <v>75</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="J22" s="21" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="G23" s="20"/>
-    </row>
-    <row r="24" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="J23" s="21"/>
+    </row>
+    <row r="24" spans="1:10" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="16"/>
-      <c r="F24" t="s">
+      <c r="E24" s="17"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="J24" s="21" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="G25" s="20"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="J25" s="21"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B26" s="12"/>
       <c r="C26" s="13"/>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="22"/>
-      <c r="F26" t="s">
+      <c r="E26" s="23"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="20"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J26" s="21"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B27" s="12"/>
-      <c r="C27" s="15"/>
+      <c r="C27" s="16"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="16" t="s">
+      <c r="E27" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="G27" s="20"/>
-    </row>
-    <row r="28" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="J27" s="21"/>
+    </row>
+    <row r="28" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E28" s="22"/>
-      <c r="F28" t="s">
+      <c r="E28" s="23"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" t="s">
         <v>44</v>
       </c>
-      <c r="G28" s="20"/>
-    </row>
-    <row r="29" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="G29" s="20"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="21" t="s">
+      <c r="J28" s="21"/>
+    </row>
+    <row r="29" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" t="s">
+        <v>113</v>
+      </c>
+      <c r="J29" s="21"/>
+    </row>
+    <row r="30" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="J30" s="21"/>
+    </row>
+    <row r="31" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" t="s">
+        <v>112</v>
+      </c>
+      <c r="J31" s="21"/>
+    </row>
+    <row r="32" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="H32" s="15"/>
+      <c r="I32" t="s">
+        <v>114</v>
+      </c>
+      <c r="J32" s="21"/>
+    </row>
+    <row r="33" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="H33" s="15"/>
+      <c r="I33" t="s">
+        <v>115</v>
+      </c>
+      <c r="J33" s="21"/>
+    </row>
+    <row r="34" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H34" s="15"/>
+      <c r="I34" t="s">
+        <v>116</v>
+      </c>
+      <c r="J34" s="21"/>
+    </row>
+    <row r="35" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="15"/>
+      <c r="I35" t="s">
+        <v>117</v>
+      </c>
+      <c r="J35" s="21"/>
+    </row>
+    <row r="36" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="H36" s="15"/>
+      <c r="I36" t="s">
+        <v>118</v>
+      </c>
+      <c r="J36" s="21"/>
+    </row>
+    <row r="37" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="J37" s="21"/>
+    </row>
+    <row r="38" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="J38" s="21"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="22"/>
-      <c r="F30" t="s">
+      <c r="E39" s="23"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" t="s">
         <v>63</v>
       </c>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="G31" s="20"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="12"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="21" t="s">
+      <c r="J39" s="21"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="J40" s="21"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="12"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E32" s="22"/>
-      <c r="F32" t="s">
+      <c r="E41" s="23"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" t="s">
         <v>47</v>
       </c>
-      <c r="G32" s="20"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="G33" s="20"/>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="12"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="21" t="s">
+      <c r="J41" s="21"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+      <c r="J42" s="21"/>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B43" s="12"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="E34" s="22"/>
-      <c r="F34" s="11" t="s">
+      <c r="E43" s="23"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="G34" s="20"/>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="20"/>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B36" s="12"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="21" t="s">
+      <c r="J43" s="21"/>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="21"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B45" s="12"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="E36" s="22"/>
-      <c r="F36" t="s">
+      <c r="E45" s="23"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+      <c r="I45" t="s">
         <v>60</v>
       </c>
-      <c r="G36" s="20"/>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="G37" s="20"/>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B38" s="12"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="21" t="s">
+      <c r="J45" s="21"/>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" s="17"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="J46" s="21"/>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B47" s="12"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="22"/>
-      <c r="F38" t="s">
+      <c r="E47" s="23"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" t="s">
         <v>56</v>
       </c>
-      <c r="G38" s="20"/>
-    </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="G39" s="20"/>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B40" s="12"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="21" t="s">
+      <c r="J47" s="21"/>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="J48" s="21"/>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B49" s="12"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="22"/>
-      <c r="G40" s="20"/>
-    </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="G41" s="20"/>
-    </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B42" s="12"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="21" t="s">
+      <c r="E49" s="23"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15"/>
+      <c r="J49" s="21"/>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
+      <c r="J50" s="21"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B51" s="12"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="22"/>
-      <c r="F42" t="s">
+      <c r="E51" s="23"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="20"/>
-    </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="G43" s="20"/>
-    </row>
-    <row r="44" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="16" t="s">
+      <c r="J51" s="21"/>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="15"/>
+      <c r="J52" s="21"/>
+    </row>
+    <row r="53" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="E44" s="16"/>
-      <c r="F44" t="s">
+      <c r="E53" s="17"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
+      <c r="I53" t="s">
         <v>84</v>
       </c>
-      <c r="G44" s="20" t="s">
+      <c r="J53" s="21" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16" t="s">
+    <row r="54" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E45" s="16"/>
-      <c r="F45" t="s">
+      <c r="E54" s="17"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" t="s">
         <v>81</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="J54" s="21" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16" t="s">
+    <row r="55" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E46" s="16"/>
-      <c r="F46" t="s">
+      <c r="E55" s="17"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
+      <c r="I55" t="s">
         <v>83</v>
       </c>
-      <c r="G46" s="20" t="s">
+      <c r="J55" s="21" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16" t="s">
+    <row r="56" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="E47" s="16"/>
-      <c r="F47" t="s">
+      <c r="E56" s="17"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" t="s">
         <v>79</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="J56" s="21" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B48" s="16"/>
-      <c r="C48" s="16" t="s">
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B57" s="17"/>
+      <c r="C57" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16"/>
-      <c r="F48" t="s">
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+      <c r="H57" s="15"/>
+      <c r="I57" t="s">
         <v>100</v>
       </c>
-      <c r="G48" s="20"/>
-    </row>
-    <row r="49" spans="2:7" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B49" s="16"/>
-      <c r="C49" s="16" t="s">
+      <c r="J57" s="21"/>
+    </row>
+    <row r="58" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B58" s="17"/>
+      <c r="C58" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
-      <c r="F49" t="s">
+      <c r="D58" s="17"/>
+      <c r="E58" s="17"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" t="s">
         <v>101</v>
       </c>
-      <c r="G49" s="19" t="s">
+      <c r="J58" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B50" s="16"/>
-      <c r="C50" s="16" t="s">
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B59" s="17"/>
+      <c r="C59" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D50" s="16"/>
-      <c r="E50" s="16"/>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="16"/>
-      <c r="C51" s="16" t="s">
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B60" s="17"/>
+      <c r="C60" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16"/>
-    </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="16"/>
-      <c r="C52" s="16" t="s">
+      <c r="D60" s="17"/>
+      <c r="E60" s="17"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61" s="17"/>
+      <c r="C61" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-    </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B53" s="16"/>
-      <c r="C53" s="16" t="s">
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B62" s="17"/>
+      <c r="C62" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D53" s="16"/>
-      <c r="E53" s="16"/>
-      <c r="F53" t="s">
+      <c r="D62" s="17"/>
+      <c r="E62" s="17"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
+      <c r="H62" s="15"/>
+      <c r="I62" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="16"/>
-      <c r="C54" s="16" t="s">
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B63" s="17"/>
+      <c r="C63" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D54" s="16"/>
-      <c r="E54" s="16"/>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B55" s="16"/>
-      <c r="C55" s="16" t="s">
+      <c r="D63" s="17"/>
+      <c r="E63" s="17"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="15"/>
+      <c r="H63" s="15"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B64" s="17"/>
+      <c r="C64" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D55" s="16"/>
-      <c r="E55" s="16"/>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B56" s="16"/>
-      <c r="C56" s="16" t="s">
+      <c r="D64" s="17"/>
+      <c r="E64" s="17"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="15"/>
+      <c r="H64" s="15"/>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B65" s="17"/>
+      <c r="C65" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D56" s="16"/>
-      <c r="E56" s="16"/>
-    </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="16"/>
-      <c r="C57" s="16" t="s">
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
+      <c r="H65" s="15"/>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B66" s="17"/>
+      <c r="C66" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D57" s="16"/>
-      <c r="E57" s="16"/>
-    </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="16"/>
-      <c r="C58" s="16" t="s">
+      <c r="D66" s="17"/>
+      <c r="E66" s="17"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="15"/>
+      <c r="H66" s="15"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B67" s="17"/>
+      <c r="C67" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D58" s="16"/>
-      <c r="E58" s="16"/>
-    </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="23"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="23"/>
-      <c r="E59" s="23"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="15"/>
+      <c r="H67" s="15"/>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B68" s="24"/>
+      <c r="C68" s="24"/>
+      <c r="D68" s="24"/>
+      <c r="E68" s="24"/>
+      <c r="F68" s="24"/>
+      <c r="G68" s="24"/>
+      <c r="H68" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update venv and evn
</commit_message>
<xml_diff>
--- a/project-structure.xlsx
+++ b/project-structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\project\pronaflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3B9866-B44E-4891-B4D9-67DEC6A26C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C010A29-8C88-4BEF-84F7-2D0E72900F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="1" xr2:uid="{159F88DC-058F-4C26-BFDD-C91DC9F7BACE}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="2" xr2:uid="{159F88DC-058F-4C26-BFDD-C91DC9F7BACE}"/>
   </bookViews>
   <sheets>
     <sheet name="Root" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="150">
   <si>
     <t>Hệ thống Tài liệu Kỹ thuật và đặc tả hệ thống</t>
   </si>
@@ -418,6 +418,78 @@
   </si>
   <si>
     <t>Toast, Loading, Skelenton</t>
+  </si>
+  <si>
+    <t>requirements.txt</t>
+  </si>
+  <si>
+    <t>Dockerfile/</t>
+  </si>
+  <si>
+    <t>tests/</t>
+  </si>
+  <si>
+    <t>main.py</t>
+  </si>
+  <si>
+    <t>__init__.py</t>
+  </si>
+  <si>
+    <t>core/</t>
+  </si>
+  <si>
+    <t>db/</t>
+  </si>
+  <si>
+    <t>base.py</t>
+  </si>
+  <si>
+    <t>mixins.py</t>
+  </si>
+  <si>
+    <t>session.py</t>
+  </si>
+  <si>
+    <t>models/</t>
+  </si>
+  <si>
+    <t>repositories/</t>
+  </si>
+  <si>
+    <t>schemas</t>
+  </si>
+  <si>
+    <t>sevices/</t>
+  </si>
+  <si>
+    <t>external/</t>
+  </si>
+  <si>
+    <t>Cấu hình chuỗi kế nối DB, Env vars</t>
+  </si>
+  <si>
+    <t>Import tất cả models vào đây để Alembic nhận diện</t>
+  </si>
+  <si>
+    <t>Khởi tạo engine AsyncIO và sessionmaker</t>
+  </si>
+  <si>
+    <t>Chứa AuditMixin và SoftDeleteMixin</t>
+  </si>
+  <si>
+    <t>Định nghĩa các SQLAlchemy Models</t>
+  </si>
+  <si>
+    <t>users.py</t>
+  </si>
+  <si>
+    <t>workspaces.py</t>
+  </si>
+  <si>
+    <t>tasks.py</t>
+  </si>
+  <si>
+    <t>enums.py</t>
   </si>
 </sst>
 </file>
@@ -529,51 +601,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -583,6 +611,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -959,13 +1029,13 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
@@ -1060,1117 +1130,1107 @@
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="11.5" style="14" customWidth="1"/>
+    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="11.5" customWidth="1"/>
     <col min="9" max="9" width="36.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="83.5" style="20" customWidth="1"/>
+    <col min="10" max="10" width="83.5" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="21">
         <v>46036</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" t="s">
         <v>24</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="12" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="17"/>
-      <c r="C9" s="17" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="17"/>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="10"/>
+      <c r="C10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
       <c r="I10" t="s">
         <v>74</v>
       </c>
-      <c r="J10" s="21"/>
+      <c r="J10" s="14"/>
     </row>
     <row r="11" spans="1:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="17" t="s">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
       <c r="I11" t="s">
         <v>66</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="14" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="17" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
       <c r="I12" t="s">
         <v>87</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="14" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="17" t="s">
+      <c r="B13" s="11"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="J13" s="21"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="J13" s="14"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="17" t="s">
+      <c r="B14" s="11"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="J14" s="21"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="J14" s="14"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="17" t="s">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
       <c r="I15" t="s">
         <v>88</v>
       </c>
-      <c r="J15" s="21" t="s">
+      <c r="J15" s="14" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="17" t="s">
+      <c r="B16" s="11"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="J16" s="21"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="17" t="s">
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="J16" s="14"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="17"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="J17" s="21"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="17" t="s">
+      <c r="E17" s="10"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="J17" s="14"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
       <c r="I18" t="s">
         <v>89</v>
       </c>
-      <c r="J18" s="21"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="17" t="s">
+      <c r="J18" s="14"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
       <c r="I19" t="s">
         <v>90</v>
       </c>
-      <c r="J19" s="21"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="14"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="17" t="s">
+      <c r="J19" s="14"/>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
       <c r="I20" t="s">
         <v>91</v>
       </c>
-      <c r="J20" s="21"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="17"/>
-      <c r="C21" s="17" t="s">
+      <c r="J20" s="14"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
       <c r="I21" t="s">
         <v>76</v>
       </c>
-      <c r="J21" s="21" t="s">
+      <c r="J21" s="14" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="12"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="17" t="s">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
       <c r="I22" t="s">
         <v>75</v>
       </c>
-      <c r="J22" s="21" t="s">
+      <c r="J22" s="14" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="J23" s="21"/>
-    </row>
-    <row r="24" spans="1:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="17" t="s">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="J23" s="14"/>
+    </row>
+    <row r="24" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B24" s="6"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="17"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
       <c r="I24" t="s">
         <v>94</v>
       </c>
-      <c r="J24" s="21" t="s">
+      <c r="J24" s="14" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="J25" s="21"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="12"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="22" t="s">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="J25" s="14"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="6"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="23"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
       <c r="I26" t="s">
         <v>58</v>
       </c>
-      <c r="J26" s="21"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="12"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="13" t="s">
+      <c r="J26" s="14"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="6"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
       <c r="I27" t="s">
         <v>124</v>
       </c>
-      <c r="J27" s="21"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="12"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="J28" s="21"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="12"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="13" t="s">
+      <c r="J27" s="14"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="6"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="J28" s="14"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="6"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
       <c r="I29" t="s">
         <v>125</v>
       </c>
-      <c r="J29" s="21"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B30" s="12"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="J30" s="21"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="12"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="J31" s="21"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="12"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="17" t="s">
+      <c r="J29" s="14"/>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="6"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="J30" s="14"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="6"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="J31" s="14"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="6"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
-      <c r="J32" s="21"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="J32" s="14"/>
     </row>
     <row r="33" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="12"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="22" t="s">
+      <c r="B33" s="6"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="23"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="15"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
       <c r="I33" t="s">
         <v>44</v>
       </c>
-      <c r="J33" s="21"/>
+      <c r="J33" s="14"/>
     </row>
     <row r="34" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17" t="s">
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
       <c r="I34" t="s">
         <v>113</v>
       </c>
-      <c r="J34" s="21"/>
+      <c r="J34" s="14"/>
     </row>
     <row r="35" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="15" t="s">
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
-      <c r="J35" s="21"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="J35" s="14"/>
     </row>
     <row r="36" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="15" t="s">
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G36" s="15"/>
-      <c r="H36" s="15"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
       <c r="I36" t="s">
         <v>112</v>
       </c>
-      <c r="J36" s="21"/>
+      <c r="J36" s="14"/>
     </row>
     <row r="37" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="15"/>
-      <c r="G37" s="15" t="s">
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="H37" s="15"/>
+      <c r="H37" s="8"/>
       <c r="I37" t="s">
         <v>114</v>
       </c>
-      <c r="J37" s="21"/>
+      <c r="J37" s="14"/>
     </row>
     <row r="38" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15" t="s">
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="H38" s="15"/>
+      <c r="H38" s="8"/>
       <c r="I38" t="s">
         <v>115</v>
       </c>
-      <c r="J38" s="21"/>
+      <c r="J38" s="14"/>
     </row>
     <row r="39" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15" t="s">
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="H39" s="15"/>
+      <c r="H39" s="8"/>
       <c r="I39" t="s">
         <v>116</v>
       </c>
-      <c r="J39" s="21"/>
+      <c r="J39" s="14"/>
     </row>
     <row r="40" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15" t="s">
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="H40" s="15"/>
+      <c r="H40" s="8"/>
       <c r="I40" t="s">
         <v>117</v>
       </c>
-      <c r="J40" s="21"/>
+      <c r="J40" s="14"/>
     </row>
     <row r="41" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15" t="s">
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="H41" s="15"/>
+      <c r="H41" s="8"/>
       <c r="I41" t="s">
         <v>118</v>
       </c>
-      <c r="J41" s="21"/>
+      <c r="J41" s="14"/>
     </row>
     <row r="42" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="15" t="s">
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
-      <c r="J42" s="21"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
+      <c r="J42" s="14"/>
     </row>
     <row r="43" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="15" t="s">
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="J43" s="21"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="J43" s="14"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="22" t="s">
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="E44" s="23"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
+      <c r="H44" s="8"/>
       <c r="I44" t="s">
         <v>63</v>
       </c>
-      <c r="J44" s="21"/>
+      <c r="J44" s="14"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="J45" s="21"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="8"/>
+      <c r="J45" s="14"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="12"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="22" t="s">
+      <c r="B46" s="6"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E46" s="23"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
       <c r="I46" t="s">
         <v>47</v>
       </c>
-      <c r="J46" s="21"/>
+      <c r="J46" s="14"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="J47" s="21"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+      <c r="J47" s="14"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B48" s="12"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="22" t="s">
+      <c r="B48" s="6"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E48" s="23"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="11" t="s">
+      <c r="E48" s="19"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="J48" s="21"/>
+      <c r="J48" s="14"/>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="12"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="13" t="s">
+      <c r="B49" s="6"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="F49" s="15"/>
-      <c r="G49" s="15"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="11"/>
-      <c r="J49" s="21"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="14"/>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="12"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="15" t="s">
+      <c r="B50" s="6"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="11" t="s">
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="J50" s="21"/>
+      <c r="J50" s="14"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="12"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="15"/>
-      <c r="I51" s="11"/>
-      <c r="J51" s="21"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="14"/>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B52" s="12"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="11"/>
-      <c r="J52" s="21"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="14"/>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B53" s="12"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="11"/>
-      <c r="J53" s="21"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="14"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="12"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="11"/>
-      <c r="J54" s="21"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="14"/>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="12"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="15"/>
-      <c r="I55" s="11"/>
-      <c r="J55" s="21"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="8"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="14"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="12"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="21"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="8"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="14"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="12"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="11"/>
-      <c r="J57" s="21"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="14"/>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="12"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-      <c r="H58" s="15"/>
-      <c r="I58" s="11"/>
-      <c r="J58" s="21"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="14"/>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="15"/>
-      <c r="I59" s="11"/>
-      <c r="J59" s="21"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="10"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="14"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="12"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="22" t="s">
+      <c r="B60" s="6"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E60" s="23"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="15"/>
+      <c r="E60" s="19"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8"/>
       <c r="I60" t="s">
         <v>60</v>
       </c>
-      <c r="J60" s="21"/>
+      <c r="J60" s="14"/>
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="17"/>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="J61" s="21"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="8"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="8"/>
+      <c r="J61" s="14"/>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B62" s="12"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="22" t="s">
+      <c r="B62" s="6"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="23"/>
-      <c r="F62" s="15"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="15"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="8"/>
+      <c r="H62" s="8"/>
       <c r="I62" t="s">
         <v>56</v>
       </c>
-      <c r="J62" s="21"/>
+      <c r="J62" s="14"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
-      <c r="H63" s="15"/>
-      <c r="J63" s="21"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="8"/>
+      <c r="G63" s="8"/>
+      <c r="H63" s="8"/>
+      <c r="J63" s="14"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="12"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="22" t="s">
+      <c r="B64" s="6"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E64" s="23"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
-      <c r="H64" s="15"/>
-      <c r="J64" s="21"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="8"/>
+      <c r="G64" s="8"/>
+      <c r="H64" s="8"/>
+      <c r="J64" s="14"/>
     </row>
     <row r="65" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B65" s="17"/>
-      <c r="C65" s="17"/>
-      <c r="D65" s="17"/>
-      <c r="E65" s="17"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
-      <c r="H65" s="15"/>
-      <c r="J65" s="21"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8"/>
+      <c r="J65" s="14"/>
     </row>
     <row r="66" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B66" s="12"/>
-      <c r="C66" s="13"/>
-      <c r="D66" s="22" t="s">
+      <c r="B66" s="6"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E66" s="23"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="15"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
       <c r="I66" t="s">
         <v>55</v>
       </c>
-      <c r="J66" s="21"/>
+      <c r="J66" s="14"/>
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B67" s="17"/>
-      <c r="C67" s="17"/>
-      <c r="D67" s="17"/>
-      <c r="E67" s="17"/>
-      <c r="F67" s="15"/>
-      <c r="G67" s="15"/>
-      <c r="H67" s="15"/>
-      <c r="J67" s="21"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="J67" s="14"/>
     </row>
     <row r="68" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B68" s="17"/>
-      <c r="C68" s="17"/>
-      <c r="D68" s="17" t="s">
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E68" s="17"/>
-      <c r="F68" s="15"/>
-      <c r="G68" s="15"/>
-      <c r="H68" s="15"/>
+      <c r="E68" s="10"/>
+      <c r="F68" s="8"/>
+      <c r="G68" s="8"/>
+      <c r="H68" s="8"/>
       <c r="I68" t="s">
         <v>84</v>
       </c>
-      <c r="J68" s="21" t="s">
+      <c r="J68" s="14" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="69" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B69" s="17"/>
-      <c r="C69" s="17"/>
-      <c r="D69" s="17" t="s">
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E69" s="17"/>
-      <c r="F69" s="15"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="15"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="8"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="8"/>
       <c r="I69" t="s">
         <v>81</v>
       </c>
-      <c r="J69" s="21" t="s">
+      <c r="J69" s="14" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="70" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17" t="s">
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E70" s="17"/>
-      <c r="F70" s="15"/>
-      <c r="G70" s="15"/>
-      <c r="H70" s="15"/>
+      <c r="E70" s="10"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8"/>
       <c r="I70" t="s">
         <v>83</v>
       </c>
-      <c r="J70" s="21" t="s">
+      <c r="J70" s="14" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="71" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B71" s="17"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17" t="s">
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E71" s="17"/>
-      <c r="F71" s="15"/>
-      <c r="G71" s="15"/>
-      <c r="H71" s="15"/>
+      <c r="E71" s="10"/>
+      <c r="F71" s="8"/>
+      <c r="G71" s="8"/>
+      <c r="H71" s="8"/>
       <c r="I71" t="s">
         <v>79</v>
       </c>
-      <c r="J71" s="21" t="s">
+      <c r="J71" s="14" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="72" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B72" s="17"/>
-      <c r="C72" s="17" t="s">
+      <c r="B72" s="10"/>
+      <c r="C72" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D72" s="17"/>
-      <c r="E72" s="17"/>
-      <c r="F72" s="15"/>
-      <c r="G72" s="15"/>
-      <c r="H72" s="15"/>
+      <c r="D72" s="10"/>
+      <c r="E72" s="10"/>
+      <c r="F72" s="8"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="8"/>
       <c r="I72" t="s">
         <v>100</v>
       </c>
-      <c r="J72" s="21"/>
+      <c r="J72" s="14"/>
     </row>
     <row r="73" spans="2:10" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="B73" s="17"/>
-      <c r="C73" s="17" t="s">
+      <c r="B73" s="10"/>
+      <c r="C73" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D73" s="17"/>
-      <c r="E73" s="17"/>
-      <c r="F73" s="15"/>
-      <c r="G73" s="15"/>
-      <c r="H73" s="15"/>
+      <c r="D73" s="10"/>
+      <c r="E73" s="10"/>
+      <c r="F73" s="8"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="8"/>
       <c r="I73" t="s">
         <v>101</v>
       </c>
-      <c r="J73" s="20" t="s">
+      <c r="J73" s="13" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="74" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B74" s="17"/>
-      <c r="C74" s="17" t="s">
+      <c r="B74" s="10"/>
+      <c r="C74" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D74" s="17"/>
-      <c r="E74" s="17"/>
-      <c r="F74" s="15"/>
-      <c r="G74" s="15"/>
-      <c r="H74" s="15"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="10"/>
+      <c r="F74" s="8"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="8"/>
     </row>
     <row r="75" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B75" s="17"/>
-      <c r="C75" s="17" t="s">
+      <c r="B75" s="10"/>
+      <c r="C75" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D75" s="17"/>
-      <c r="E75" s="17"/>
-      <c r="F75" s="15"/>
-      <c r="G75" s="15"/>
-      <c r="H75" s="15"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10"/>
+      <c r="F75" s="8"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="8"/>
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B76" s="17"/>
-      <c r="C76" s="17" t="s">
+      <c r="B76" s="10"/>
+      <c r="C76" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D76" s="17"/>
-      <c r="E76" s="17"/>
-      <c r="F76" s="15"/>
-      <c r="G76" s="15"/>
-      <c r="H76" s="15"/>
+      <c r="D76" s="10"/>
+      <c r="E76" s="10"/>
+      <c r="F76" s="8"/>
+      <c r="G76" s="8"/>
+      <c r="H76" s="8"/>
     </row>
     <row r="77" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B77" s="17"/>
-      <c r="C77" s="17" t="s">
+      <c r="B77" s="10"/>
+      <c r="C77" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D77" s="17"/>
-      <c r="E77" s="17"/>
-      <c r="F77" s="15"/>
-      <c r="G77" s="15"/>
-      <c r="H77" s="15"/>
+      <c r="D77" s="10"/>
+      <c r="E77" s="10"/>
+      <c r="F77" s="8"/>
+      <c r="G77" s="8"/>
+      <c r="H77" s="8"/>
       <c r="I77" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B78" s="17"/>
-      <c r="C78" s="17" t="s">
+      <c r="B78" s="10"/>
+      <c r="C78" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D78" s="17"/>
-      <c r="E78" s="17"/>
-      <c r="F78" s="15"/>
-      <c r="G78" s="15"/>
-      <c r="H78" s="15"/>
+      <c r="D78" s="10"/>
+      <c r="E78" s="10"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="8"/>
+      <c r="H78" s="8"/>
     </row>
     <row r="79" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B79" s="17"/>
-      <c r="C79" s="17" t="s">
+      <c r="B79" s="10"/>
+      <c r="C79" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D79" s="17"/>
-      <c r="E79" s="17"/>
-      <c r="F79" s="15"/>
-      <c r="G79" s="15"/>
-      <c r="H79" s="15"/>
+      <c r="D79" s="10"/>
+      <c r="E79" s="10"/>
+      <c r="F79" s="8"/>
+      <c r="G79" s="8"/>
+      <c r="H79" s="8"/>
     </row>
     <row r="80" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B80" s="17"/>
-      <c r="C80" s="17" t="s">
+      <c r="B80" s="10"/>
+      <c r="C80" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D80" s="17"/>
-      <c r="E80" s="17"/>
-      <c r="F80" s="15"/>
-      <c r="G80" s="15"/>
-      <c r="H80" s="15"/>
+      <c r="D80" s="10"/>
+      <c r="E80" s="10"/>
+      <c r="F80" s="8"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="8"/>
     </row>
     <row r="81" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B81" s="17"/>
-      <c r="C81" s="17" t="s">
+      <c r="B81" s="10"/>
+      <c r="C81" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D81" s="17"/>
-      <c r="E81" s="17"/>
-      <c r="F81" s="15"/>
-      <c r="G81" s="15"/>
-      <c r="H81" s="15"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="10"/>
+      <c r="F81" s="8"/>
+      <c r="G81" s="8"/>
+      <c r="H81" s="8"/>
     </row>
     <row r="82" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B82" s="17"/>
-      <c r="C82" s="17" t="s">
+      <c r="B82" s="10"/>
+      <c r="C82" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D82" s="17"/>
-      <c r="E82" s="17"/>
-      <c r="F82" s="15"/>
-      <c r="G82" s="15"/>
-      <c r="H82" s="15"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="10"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="8"/>
+      <c r="H82" s="8"/>
     </row>
     <row r="83" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B83" s="24"/>
-      <c r="C83" s="24"/>
-      <c r="D83" s="24"/>
-      <c r="E83" s="24"/>
-      <c r="F83" s="24"/>
-      <c r="G83" s="24"/>
-      <c r="H83" s="24"/>
+      <c r="B83" s="8"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="8"/>
+      <c r="E83" s="8"/>
+      <c r="F83" s="8"/>
+      <c r="G83" s="8"/>
+      <c r="H83" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B1:J1"/>
     <mergeCell ref="D64:E64"/>
     <mergeCell ref="D66:E66"/>
     <mergeCell ref="D26:E26"/>
@@ -2178,11 +2238,11 @@
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D46:E46"/>
     <mergeCell ref="D48:E48"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D62:E62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2190,9 +2250,997 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8EBE1E2-9900-4FFB-890F-7B8D2A7D702D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="11.5" customWidth="1"/>
+    <col min="9" max="9" width="36.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="83.5" style="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="21">
+        <v>46036</v>
+      </c>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="10"/>
+      <c r="C9" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="10"/>
+      <c r="C10" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="J10" s="14"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="J11" s="14"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E12" s="10"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="J12" s="14"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="11"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="J13" s="14"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="11"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="J14" s="14"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" t="s">
+        <v>141</v>
+      </c>
+      <c r="J15" s="14"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="J16" s="14"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="J17" s="14"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" t="s">
+        <v>142</v>
+      </c>
+      <c r="J18" s="14"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J19" s="14"/>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" t="s">
+        <v>143</v>
+      </c>
+      <c r="J20" s="14"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="E21" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" t="s">
+        <v>145</v>
+      </c>
+      <c r="J21" s="14"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="J22" s="14"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="6"/>
+      <c r="C23" s="7"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="J23" s="14"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="6"/>
+      <c r="C24" s="7"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="J24" s="14"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="J25" s="14"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="6"/>
+      <c r="C26" s="7"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="J26" s="14"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="6"/>
+      <c r="C27" s="7"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="J27" s="14"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="6"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="J28" s="14"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E29" s="10"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="J29" s="14"/>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="6"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="J30" s="14"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="J31" s="14"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="6"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="J32" s="14"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B33" s="6"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="J33" s="14"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" s="6"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="J34" s="14"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="6"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="J35" s="14"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" s="6"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="J36" s="14"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" s="6"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="J37" s="14"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B38" s="6"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="J38" s="14"/>
+    </row>
+    <row r="39" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="6"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="J39" s="14"/>
+    </row>
+    <row r="40" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="10"/>
+      <c r="C40" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="J40" s="14"/>
+    </row>
+    <row r="41" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="10"/>
+      <c r="C41" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D41" s="6"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="8"/>
+      <c r="J41" s="14"/>
+    </row>
+    <row r="42" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
+      <c r="J42" s="14"/>
+    </row>
+    <row r="43" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="J43" s="14"/>
+    </row>
+    <row r="44" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
+      <c r="H44" s="8"/>
+      <c r="J44" s="14"/>
+    </row>
+    <row r="45" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="8"/>
+      <c r="J45" s="14"/>
+    </row>
+    <row r="46" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
+      <c r="J46" s="14"/>
+    </row>
+    <row r="47" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+      <c r="J47" s="14"/>
+    </row>
+    <row r="48" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="J48" s="14"/>
+    </row>
+    <row r="49" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="J49" s="14"/>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="J50" s="14"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+      <c r="J51" s="14"/>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B52" s="6"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="J52" s="14"/>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="J53" s="14"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B54" s="6"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="14"/>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B55" s="6"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="8"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="14"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B56" s="6"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="8"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="14"/>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B57" s="6"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="14"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B58" s="6"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="14"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B59" s="6"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="14"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B60" s="6"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="14"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61" s="6"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="8"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="8"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="14"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B62" s="6"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="8"/>
+      <c r="H62" s="8"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="14"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B63" s="6"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="8"/>
+      <c r="G63" s="8"/>
+      <c r="H63" s="8"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="14"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B64" s="6"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="8"/>
+      <c r="G64" s="8"/>
+      <c r="H64" s="8"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="14"/>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8"/>
+      <c r="I65" s="5"/>
+      <c r="J65" s="14"/>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B66" s="6"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
+      <c r="J66" s="14"/>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="J67" s="14"/>
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B68" s="6"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="18"/>
+      <c r="E68" s="19"/>
+      <c r="F68" s="8"/>
+      <c r="G68" s="8"/>
+      <c r="H68" s="8"/>
+      <c r="J68" s="14"/>
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="8"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="8"/>
+      <c r="J69" s="14"/>
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B70" s="6"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8"/>
+      <c r="J70" s="14"/>
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="10"/>
+      <c r="E71" s="10"/>
+      <c r="F71" s="8"/>
+      <c r="G71" s="8"/>
+      <c r="H71" s="8"/>
+      <c r="J71" s="14"/>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B72" s="6"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="19"/>
+      <c r="F72" s="8"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="8"/>
+      <c r="J72" s="14"/>
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="10"/>
+      <c r="E73" s="10"/>
+      <c r="F73" s="8"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="8"/>
+      <c r="J73" s="14"/>
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="10"/>
+      <c r="F74" s="8"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="8"/>
+      <c r="J74" s="14"/>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10"/>
+      <c r="F75" s="8"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="8"/>
+      <c r="J75" s="14"/>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10"/>
+      <c r="E76" s="10"/>
+      <c r="F76" s="8"/>
+      <c r="G76" s="8"/>
+      <c r="H76" s="8"/>
+      <c r="J76" s="14"/>
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="10"/>
+      <c r="E77" s="10"/>
+      <c r="F77" s="8"/>
+      <c r="G77" s="8"/>
+      <c r="H77" s="8"/>
+      <c r="J77" s="14"/>
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10"/>
+      <c r="E78" s="10"/>
+      <c r="F78" s="8"/>
+      <c r="G78" s="8"/>
+      <c r="H78" s="8"/>
+      <c r="J78" s="14"/>
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="10"/>
+      <c r="E79" s="10"/>
+      <c r="F79" s="8"/>
+      <c r="G79" s="8"/>
+      <c r="H79" s="8"/>
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="10"/>
+      <c r="E80" s="10"/>
+      <c r="F80" s="8"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="8"/>
+    </row>
+    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="10"/>
+      <c r="F81" s="8"/>
+      <c r="G81" s="8"/>
+      <c r="H81" s="8"/>
+    </row>
+    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="10"/>
+      <c r="F82" s="8"/>
+      <c r="G82" s="8"/>
+      <c r="H82" s="8"/>
+    </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B83" s="10"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="10"/>
+      <c r="E83" s="10"/>
+      <c r="F83" s="8"/>
+      <c r="G83" s="8"/>
+      <c r="H83" s="8"/>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B84" s="10"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="10"/>
+      <c r="E84" s="10"/>
+      <c r="F84" s="8"/>
+      <c r="G84" s="8"/>
+      <c r="H84" s="8"/>
+    </row>
+    <row r="85" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="10"/>
+      <c r="E85" s="10"/>
+      <c r="F85" s="8"/>
+      <c r="G85" s="8"/>
+      <c r="H85" s="8"/>
+    </row>
+    <row r="86" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="10"/>
+      <c r="F86" s="8"/>
+      <c r="G86" s="8"/>
+      <c r="H86" s="8"/>
+    </row>
+    <row r="87" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B87" s="10"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="10"/>
+      <c r="E87" s="10"/>
+      <c r="F87" s="8"/>
+      <c r="G87" s="8"/>
+      <c r="H87" s="8"/>
+    </row>
+    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B88" s="10"/>
+      <c r="C88" s="10"/>
+      <c r="D88" s="10"/>
+      <c r="E88" s="10"/>
+      <c r="F88" s="8"/>
+      <c r="G88" s="8"/>
+      <c r="H88" s="8"/>
+    </row>
+    <row r="89" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B89" s="8"/>
+      <c r="C89" s="8"/>
+      <c r="D89" s="8"/>
+      <c r="E89" s="8"/>
+      <c r="F89" s="8"/>
+      <c r="G89" s="8"/>
+      <c r="H89" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="A6:J6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>